<commit_message>
Linking groups to educational programs
</commit_message>
<xml_diff>
--- a/chm_choice_of_practices/static/templates/шаблон_звіту_поточного_підприємства.xlsx
+++ b/chm_choice_of_practices/static/templates/шаблон_звіту_поточного_підприємства.xlsx
@@ -1185,53 +1185,53 @@
     <xf numFmtId="0" fontId="47" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="45" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="46" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="47" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1635,7 +1635,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1659,53 +1659,53 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
     </row>
     <row r="2" spans="1:8" ht="22.8">
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
     </row>
     <row r="3" spans="1:8" ht="15.6">
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
-      <c r="H3" s="20"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21"/>
     </row>
     <row r="4" spans="1:8" ht="15.45" customHeight="1">
       <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="14"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
     </row>
     <row r="5" spans="1:8" ht="15.6">
-      <c r="B5" s="21"/>
-      <c r="C5" s="21"/>
-      <c r="D5" s="21"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="21"/>
+      <c r="B5" s="23"/>
+      <c r="C5" s="23"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="23"/>
+      <c r="F5" s="23"/>
       <c r="G5" s="3" t="s">
         <v>2</v>
       </c>
@@ -1717,170 +1717,170 @@
       <c r="B6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="14"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="22"/>
     </row>
     <row r="7" spans="1:8">
       <c r="B7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="22"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="22"/>
     </row>
     <row r="8" spans="1:8">
       <c r="B8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="C8" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
+      <c r="D8" s="22"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="22"/>
+      <c r="G8" s="22"/>
+      <c r="H8" s="22"/>
     </row>
     <row r="9" spans="1:8">
       <c r="B9" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="C9" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="22"/>
+      <c r="H9" s="22"/>
     </row>
     <row r="10" spans="1:8">
       <c r="B10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="22"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="22"/>
     </row>
     <row r="11" spans="1:8">
       <c r="B11" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14"/>
-      <c r="F11" s="14"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
+      <c r="G11" s="22"/>
+      <c r="H11" s="22"/>
     </row>
     <row r="12" spans="1:8">
       <c r="B12" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="22"/>
+      <c r="H12" s="22"/>
     </row>
     <row r="13" spans="1:8">
       <c r="B13" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="C13" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
+      <c r="G13" s="22"/>
+      <c r="H13" s="22"/>
     </row>
     <row r="14" spans="1:8" ht="15.6">
       <c r="A14" s="2"/>
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
-      <c r="G14" s="15"/>
-      <c r="H14" s="15"/>
+      <c r="C14" s="26"/>
+      <c r="D14" s="26"/>
+      <c r="E14" s="26"/>
+      <c r="F14" s="26"/>
+      <c r="G14" s="26"/>
+      <c r="H14" s="26"/>
     </row>
     <row r="15" spans="1:8">
       <c r="B15" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="26" t="s">
+      <c r="C15" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="D15" s="26" t="s">
+      <c r="D15" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="E15" s="26" t="s">
+      <c r="E15" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="F15" s="16" t="s">
+      <c r="F15" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="G15" s="16"/>
-      <c r="H15" s="26" t="s">
+      <c r="G15" s="27"/>
+      <c r="H15" s="12" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:8">
-      <c r="B16" s="27" t="s">
+      <c r="B16" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="C16" s="27" t="s">
+      <c r="C16" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="D16" s="27" t="s">
+      <c r="D16" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="E16" s="27" t="s">
+      <c r="E16" s="13" t="s">
         <v>42</v>
       </c>
       <c r="F16" s="28" t="s">
         <v>43</v>
       </c>
       <c r="G16" s="29"/>
-      <c r="H16" s="27" t="s">
+      <c r="H16" s="13" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:8">
-      <c r="B17" s="12" t="s">
+      <c r="B17" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="13"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="13"/>
-      <c r="H17" s="13"/>
+      <c r="C17" s="25"/>
+      <c r="D17" s="25"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="25"/>
+      <c r="G17" s="25"/>
+      <c r="H17" s="25"/>
     </row>
     <row r="18" spans="1:8">
       <c r="B18" s="5" t="s">
@@ -1896,10 +1896,10 @@
         <v>28</v>
       </c>
       <c r="F18" s="9"/>
-      <c r="G18" s="22" t="s">
+      <c r="G18" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="H18" s="23"/>
+      <c r="H18" s="15"/>
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="1" t="s">
@@ -1918,10 +1918,10 @@
         <v>37</v>
       </c>
       <c r="F19" s="6"/>
-      <c r="G19" s="24" t="s">
+      <c r="G19" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="H19" s="25"/>
+      <c r="H19" s="17"/>
     </row>
     <row r="20" spans="1:8">
       <c r="A20" s="1" t="s">
@@ -1936,11 +1936,15 @@
       <c r="D20" s="8"/>
       <c r="E20" s="8"/>
       <c r="F20" s="10"/>
-      <c r="G20" s="24"/>
-      <c r="H20" s="25"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="C13:H13"/>
+    <mergeCell ref="B14:H14"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="F16:G16"/>
     <mergeCell ref="G18:H18"/>
     <mergeCell ref="G19:H19"/>
     <mergeCell ref="G20:H20"/>
@@ -1957,10 +1961,6 @@
     <mergeCell ref="C10:H10"/>
     <mergeCell ref="C11:H11"/>
     <mergeCell ref="C12:H12"/>
-    <mergeCell ref="C13:H13"/>
-    <mergeCell ref="B14:H14"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="F16:G16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>